<commit_message>
consolidado limpio y codigo actualizado
</commit_message>
<xml_diff>
--- a/consolidado_limpio.xlsx
+++ b/consolidado_limpio.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,41 +464,6 @@
           <t>metodo_pago</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha_Venta</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Categoria</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Cant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Valor_Unitario</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Vendedor</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -532,13 +497,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -572,13 +530,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -612,13 +563,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,13 +596,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -692,13 +629,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,13 +662,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -767,14 +690,11 @@
           <t>Laura Diaz</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -808,13 +728,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -848,13 +761,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -888,13 +794,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -923,14 +822,11 @@
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -964,13 +860,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1004,13 +893,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1039,14 +921,11 @@
           <t>Laura Diaz</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1080,13 +959,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1120,13 +992,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1155,14 +1020,11 @@
           <t>Sofia Mena</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1196,13 +1058,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1236,13 +1091,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1276,13 +1124,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1316,13 +1157,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1356,13 +1190,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1391,14 +1218,11 @@
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1432,13 +1256,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1472,13 +1289,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1512,13 +1322,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1547,14 +1350,11 @@
           <t>Laura Diaz</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1588,13 +1388,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1628,13 +1421,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1668,13 +1454,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1703,14 +1482,11 @@
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1739,14 +1515,11 @@
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1780,13 +1553,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1820,13 +1586,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1847,7 +1606,9 @@
       <c r="D36" t="n">
         <v>6</v>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>Felipe Torres</t>
@@ -1858,13 +1619,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1898,13 +1652,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1928,19 +1675,16 @@
       <c r="E38" t="n">
         <v>34000</v>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1974,13 +1718,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2014,13 +1751,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2041,7 +1771,9 @@
       <c r="D41" t="n">
         <v>1</v>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>Andres Gomez</t>
@@ -2052,13 +1784,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2092,13 +1817,6 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2122,19 +1840,16 @@
       <c r="E43" t="n">
         <v>152700</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2168,13 +1883,6 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2195,20 +1903,19 @@
       <c r="D45" t="n">
         <v>4</v>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>Laura Diaz</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2237,14 +1944,11 @@
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2278,13 +1982,6 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2313,14 +2010,11 @@
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2354,601 +2048,501 @@
           <t>Tarjeta</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Medias deportivas</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K50" t="n">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
         <v>7</v>
       </c>
-      <c r="L50" t="n">
+      <c r="E50" t="n">
         <v>78000</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Felipe Torres</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Parlante portatil</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Electronica</t>
-        </is>
-      </c>
-      <c r="K51" t="n">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
         <v>2</v>
       </c>
-      <c r="L51" t="n">
+      <c r="E51" t="n">
         <v>127500</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Sofia Mena</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>Chaqueta impermeable</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K52" t="n">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
         <v>5</v>
       </c>
-      <c r="L52" t="n">
+      <c r="E52" t="n">
         <v>86700</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Felipe Torres</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Cargador USB-C</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Electronica</t>
-        </is>
-      </c>
-      <c r="K53" t="n">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
         <v>3</v>
       </c>
-      <c r="L53" t="n">
+      <c r="E53" t="n">
         <v>98800</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Parlante portatil</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Electronica</t>
-        </is>
-      </c>
-      <c r="K54" t="n">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
         <v>4</v>
       </c>
-      <c r="L54" t="n">
+      <c r="E54" t="n">
         <v>40200</v>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Medias deportivas</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K55" t="n">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
         <v>8</v>
       </c>
-      <c r="L55" t="n">
+      <c r="E55" t="n">
         <v>18200</v>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Laura Diaz</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Jean clasico</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K56" t="n">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
         <v>4</v>
       </c>
-      <c r="L56" t="n">
+      <c r="E56" t="n">
         <v>159900</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Gorra deportiva</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K57" t="n">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
         <v>3</v>
       </c>
-      <c r="L57" t="n">
+      <c r="E57" t="n">
         <v>36200</v>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>Felipe Torres</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Cargador USB-C</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Electronica</t>
-        </is>
-      </c>
-      <c r="K58" t="n">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
         <v>7</v>
       </c>
-      <c r="L58" t="n">
+      <c r="E58" t="n">
         <v>174100</v>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>Sofia Mena</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Cargador USB-C</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Electronica</t>
-        </is>
-      </c>
-      <c r="K59" t="n">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
         <v>6</v>
       </c>
-      <c r="L59" t="n">
+      <c r="E59" t="n">
         <v>87300</v>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Sofia Mena</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Camiseta basica</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K60" t="n">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
         <v>4</v>
       </c>
-      <c r="L60" t="n">
+      <c r="E60" t="n">
         <v>25600</v>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Medias deportivas</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K61" t="n">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
         <v>1</v>
       </c>
-      <c r="L61" t="n">
+      <c r="E61" t="n">
         <v>26700</v>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Camiseta basica</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K62" t="n">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
         <v>6</v>
       </c>
-      <c r="L62" t="n">
+      <c r="E62" t="n">
         <v>26700</v>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Gorra deportiva</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K63" t="n">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
         <v>3</v>
       </c>
-      <c r="L63" t="n">
+      <c r="E63" t="n">
         <v>134400</v>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Sofia Mena</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>Jean clasico</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="K64" t="n">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
         <v>7</v>
       </c>
-      <c r="L64" t="n">
+      <c r="E64" t="n">
         <v>46400</v>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>